<commit_message>
Projeto do showroom em 58 módulos com a spec de peças de 10/09
- analise/showroom-projeto.py posiciona os 58 módulos na planta e aloca o
  catálogo módulo a módulo: 605 de 609 SKUs (99,5% do faturamento), ilhas
  recebem as sobras das paredes, campeões repetem em pontas e checkout.
- dados/55 módulos posicionados, 56 alocação SKU a SKU, 57 lista de compras.
- analise/18-projeto-showroom.html: planta baixa, elevações das quatro
  paredes, módulos-tipo, compras, ancoragem e as três fitas a conferir.
- plano-pecas: laterais de 372 mudam o fundo para 8x759 + 1x659
  (58 módulos, R$ 15.657, 854 kg); dados/54 regenerado.
- CLAUDE.md registra a composição nova e as conclusões do projeto.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WcfaWwNy7qc1Kvnvnn813R
</commit_message>
<xml_diff>
--- a/dados/54-plano-pecas.xlsx
+++ b/dados/54-plano-pecas.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="152">
   <si>
     <t xml:space="preserve">Nitron Mob PDV — as peças (lista de 10/09/2026)</t>
   </si>
@@ -334,6 +334,12 @@
     <t xml:space="preserve">Parede do fundo · lixeira na baia de 490 e nas duas de 323; olhos a 1.542</t>
   </si>
   <si>
+    <t xml:space="preserve">fundo-620</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parede do fundo · ajuste de canto, mesma pilha</t>
+  </si>
+  <si>
     <t xml:space="preserve">ponta</t>
   </si>
   <si>
@@ -373,7 +379,7 @@
     <t xml:space="preserve">O showroom com as peças novas — onde vai cada módulo e quanto</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantidades em azul são a proposta; troque e o resto recalcula. Paredes: 14 × 759 + 4 × 659 no sul (folga 88), 8 × 759 no norte (28), 9 × 759 no fundo (42). Entrada: 3 módulos + vitrine.</t>
+    <t xml:space="preserve">Quantidades em azul são a proposta; troque e o resto recalcula. Paredes: sul 14 × 759 + 4 × 659 (folga 88) · norte 8 × 759 (161) · fundo 8 × 759 + 1 × 659 (45) · entrada 3 módulos + vitrine de 2871 mm.</t>
   </si>
   <si>
     <t xml:space="preserve">Onde</t>
@@ -401,6 +407,9 @@
   </si>
   <si>
     <t xml:space="preserve">Paredão do fundo · banho e lavanderia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paredão do fundo · ajuste de canto</t>
   </si>
   <si>
     <t xml:space="preserve">Parede de entrada · frasqueiras e infantil</t>
@@ -1340,7 +1349,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:X11"/>
+  <dimension ref="A1:X12"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -1707,39 +1716,39 @@
         <v>103</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>287</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>717</v>
+        <v>617</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">F8+1</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>759</v>
+        <v>659</v>
       </c>
       <c r="J8" s="11" t="n">
         <v>372.3</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>1030.1</v>
+        <v>1535</v>
       </c>
       <c r="L8" s="10" t="n">
         <f aca="false">4*H8</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="M8" s="10" t="n">
         <f aca="false">IF(G8&gt;0,4,0)</f>
@@ -1750,15 +1759,15 @@
       </c>
       <c r="O8" s="10" t="n">
         <f aca="false">H8</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P8" s="10" t="n">
         <f aca="false">2*(H8+IF(G8&gt;0,1,0))</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q8" s="10" t="n">
         <f aca="false">2*H8</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R8" s="10" t="n">
         <f aca="false">4*1</f>
@@ -1769,62 +1778,62 @@
         <v>8</v>
       </c>
       <c r="T8" s="10" t="n">
-        <f aca="false">4*0</f>
-        <v>0</v>
+        <f aca="false">4*1</f>
+        <v>4</v>
       </c>
       <c r="U8" s="10" t="n">
         <v>4</v>
       </c>
       <c r="V8" s="12" t="n">
-        <f aca="false">L8*Pecas!$D$18+M8*Pecas!$D$20+N8*Pecas!$D$21+O8*Pecas!$D$7+P8*Pecas!$D$13+Q8*Pecas!$D$10+R8*Pecas!$D$14+S8*Pecas!$D$15+T8*Pecas!$D$16+U8*Pecas!$D$17</f>
-        <v>10.832</v>
+        <f aca="false">L8*Pecas!$D$18+M8*Pecas!$D$20+N8*Pecas!$D$21+O8*Pecas!$D$6+P8*Pecas!$D$12+Q8*Pecas!$D$10+R8*Pecas!$D$14+S8*Pecas!$D$15+T8*Pecas!$D$16+U8*Pecas!$D$17</f>
+        <v>12.2105</v>
       </c>
       <c r="W8" s="13" t="n">
-        <f aca="false">L8*Pecas!$E$18+M8*Pecas!$E$20+N8*Pecas!$E$21+O8*Pecas!$E$7+P8*Pecas!$E$13+Q8*Pecas!$E$10+R8*Pecas!$E$14+S8*Pecas!$E$15+T8*Pecas!$E$16+U8*Pecas!$E$17</f>
-        <v>198.8084</v>
+        <f aca="false">L8*Pecas!$E$18+M8*Pecas!$E$20+N8*Pecas!$E$21+O8*Pecas!$E$6+P8*Pecas!$E$12+Q8*Pecas!$E$10+R8*Pecas!$E$14+S8*Pecas!$E$15+T8*Pecas!$E$16+U8*Pecas!$E$17</f>
+        <v>223.2165</v>
       </c>
       <c r="X8" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>415</v>
+        <v>287</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>717</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">F9+1</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I9" s="11" t="n">
         <v>759</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>500.3</v>
+        <v>372.3</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>935.2</v>
+        <v>1030.1</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">4*H9</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="M9" s="10" t="n">
         <f aca="false">IF(G9&gt;0,4,0)</f>
@@ -1835,81 +1844,81 @@
       </c>
       <c r="O9" s="10" t="n">
         <f aca="false">H9</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" s="10" t="n">
         <f aca="false">2*(H9+IF(G9&gt;0,1,0))</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q9" s="10" t="n">
         <f aca="false">2*H9</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R9" s="10" t="n">
+        <f aca="false">4*1</f>
+        <v>4</v>
+      </c>
+      <c r="S9" s="10" t="n">
+        <f aca="false">4*2</f>
+        <v>8</v>
+      </c>
+      <c r="T9" s="10" t="n">
         <f aca="false">4*0</f>
         <v>0</v>
       </c>
-      <c r="S9" s="10" t="n">
-        <f aca="false">4*1</f>
-        <v>4</v>
-      </c>
-      <c r="T9" s="10" t="n">
-        <f aca="false">4*1</f>
-        <v>4</v>
-      </c>
       <c r="U9" s="10" t="n">
         <v>4</v>
       </c>
       <c r="V9" s="12" t="n">
-        <f aca="false">L9*Pecas!$D$18+M9*Pecas!$D$20+N9*Pecas!$D$21+O9*Pecas!$D$8+P9*Pecas!$D$13+Q9*Pecas!$D$11+R9*Pecas!$D$14+S9*Pecas!$D$15+T9*Pecas!$D$16+U9*Pecas!$D$17</f>
-        <v>11.0673</v>
+        <f aca="false">L9*Pecas!$D$18+M9*Pecas!$D$20+N9*Pecas!$D$21+O9*Pecas!$D$7+P9*Pecas!$D$13+Q9*Pecas!$D$10+R9*Pecas!$D$14+S9*Pecas!$D$15+T9*Pecas!$D$16+U9*Pecas!$D$17</f>
+        <v>10.832</v>
       </c>
       <c r="W9" s="13" t="n">
-        <f aca="false">L9*Pecas!$E$18+M9*Pecas!$E$20+N9*Pecas!$E$21+O9*Pecas!$E$8+P9*Pecas!$E$13+Q9*Pecas!$E$11+R9*Pecas!$E$14+S9*Pecas!$E$15+T9*Pecas!$E$16+U9*Pecas!$E$17</f>
-        <v>205.1026</v>
+        <f aca="false">L9*Pecas!$E$18+M9*Pecas!$E$20+N9*Pecas!$E$21+O9*Pecas!$E$7+P9*Pecas!$E$13+Q9*Pecas!$E$10+R9*Pecas!$E$14+S9*Pecas!$E$15+T9*Pecas!$E$16+U9*Pecas!$E$17</f>
+        <v>198.8084</v>
       </c>
       <c r="X9" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>415</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>717</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="9" t="n">
-        <v>183</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>617</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>110</v>
-      </c>
       <c r="F10" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">F10+1</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>659</v>
+        <v>759</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>268.3</v>
+        <v>500.3</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>878.1</v>
+        <v>935.2</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">4*H10</f>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="M10" s="10" t="n">
         <f aca="false">IF(G10&gt;0,4,0)</f>
@@ -1920,92 +1929,92 @@
       </c>
       <c r="O10" s="10" t="n">
         <f aca="false">H10</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P10" s="10" t="n">
         <f aca="false">2*(H10+IF(G10&gt;0,1,0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="10" t="n">
         <f aca="false">2*H10</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R10" s="10" t="n">
-        <f aca="false">4*3</f>
-        <v>12</v>
-      </c>
-      <c r="S10" s="10" t="n">
         <f aca="false">4*0</f>
         <v>0</v>
       </c>
+      <c r="S10" s="10" t="n">
+        <f aca="false">4*1</f>
+        <v>4</v>
+      </c>
       <c r="T10" s="10" t="n">
-        <f aca="false">4*0</f>
-        <v>0</v>
+        <f aca="false">4*1</f>
+        <v>4</v>
       </c>
       <c r="U10" s="10" t="n">
         <v>4</v>
       </c>
       <c r="V10" s="12" t="n">
-        <f aca="false">L10*Pecas!$D$18+M10*Pecas!$D$20+N10*Pecas!$D$21+O10*Pecas!$D$5+P10*Pecas!$D$12+Q10*Pecas!$D$9+R10*Pecas!$D$14+S10*Pecas!$D$15+T10*Pecas!$D$16+U10*Pecas!$D$17</f>
-        <v>7.0856</v>
+        <f aca="false">L10*Pecas!$D$18+M10*Pecas!$D$20+N10*Pecas!$D$21+O10*Pecas!$D$8+P10*Pecas!$D$13+Q10*Pecas!$D$11+R10*Pecas!$D$14+S10*Pecas!$D$15+T10*Pecas!$D$16+U10*Pecas!$D$17</f>
+        <v>11.0673</v>
       </c>
       <c r="W10" s="13" t="n">
-        <f aca="false">L10*Pecas!$E$18+M10*Pecas!$E$20+N10*Pecas!$E$21+O10*Pecas!$E$5+P10*Pecas!$E$12+Q10*Pecas!$E$9+R10*Pecas!$E$14+S10*Pecas!$E$15+T10*Pecas!$E$16+U10*Pecas!$E$17</f>
-        <v>127.5032</v>
+        <f aca="false">L10*Pecas!$E$18+M10*Pecas!$E$20+N10*Pecas!$E$21+O10*Pecas!$E$8+P10*Pecas!$E$13+Q10*Pecas!$E$11+R10*Pecas!$E$14+S10*Pecas!$E$15+T10*Pecas!$E$16+U10*Pecas!$E$17</f>
+        <v>205.1026</v>
       </c>
       <c r="X10" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>183</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>617</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C11" s="9" t="n">
-        <v>287</v>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>717</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>113</v>
-      </c>
       <c r="F11" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>513</v>
+        <v>0</v>
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">F11+1</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>759</v>
+        <v>659</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>372.3</v>
+        <v>268.3</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>1607.1</v>
+        <v>878.1</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">4*H11</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="M11" s="10" t="n">
         <f aca="false">IF(G11&gt;0,4,0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>4</v>
       </c>
       <c r="O11" s="10" t="n">
         <f aca="false">H11</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P11" s="10" t="n">
         <f aca="false">2*(H11+IF(G11&gt;0,1,0))</f>
@@ -2013,33 +2022,118 @@
       </c>
       <c r="Q11" s="10" t="n">
         <f aca="false">2*H11</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R11" s="10" t="n">
-        <f aca="false">4*0</f>
-        <v>0</v>
+        <f aca="false">4*3</f>
+        <v>12</v>
       </c>
       <c r="S11" s="10" t="n">
         <f aca="false">4*0</f>
         <v>0</v>
       </c>
       <c r="T11" s="10" t="n">
+        <f aca="false">4*0</f>
+        <v>0</v>
+      </c>
+      <c r="U11" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="V11" s="12" t="n">
+        <f aca="false">L11*Pecas!$D$18+M11*Pecas!$D$20+N11*Pecas!$D$21+O11*Pecas!$D$5+P11*Pecas!$D$12+Q11*Pecas!$D$9+R11*Pecas!$D$14+S11*Pecas!$D$15+T11*Pecas!$D$16+U11*Pecas!$D$17</f>
+        <v>7.0856</v>
+      </c>
+      <c r="W11" s="13" t="n">
+        <f aca="false">L11*Pecas!$E$18+M11*Pecas!$E$20+N11*Pecas!$E$21+O11*Pecas!$E$5+P11*Pecas!$E$12+Q11*Pecas!$E$9+R11*Pecas!$E$14+S11*Pecas!$E$15+T11*Pecas!$E$16+U11*Pecas!$E$17</f>
+        <v>127.5032</v>
+      </c>
+      <c r="X11" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>287</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>717</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>513</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <f aca="false">F12+1</f>
+        <v>3</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>759</v>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>372.3</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <v>1607.1</v>
+      </c>
+      <c r="L12" s="10" t="n">
+        <f aca="false">4*H12</f>
+        <v>12</v>
+      </c>
+      <c r="M12" s="10" t="n">
+        <f aca="false">IF(G12&gt;0,4,0)</f>
+        <v>4</v>
+      </c>
+      <c r="N12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="O12" s="10" t="n">
+        <f aca="false">H12</f>
+        <v>3</v>
+      </c>
+      <c r="P12" s="10" t="n">
+        <f aca="false">2*(H12+IF(G12&gt;0,1,0))</f>
+        <v>8</v>
+      </c>
+      <c r="Q12" s="10" t="n">
+        <f aca="false">2*H12</f>
+        <v>6</v>
+      </c>
+      <c r="R12" s="10" t="n">
+        <f aca="false">4*0</f>
+        <v>0</v>
+      </c>
+      <c r="S12" s="10" t="n">
+        <f aca="false">4*0</f>
+        <v>0</v>
+      </c>
+      <c r="T12" s="10" t="n">
         <f aca="false">4*3</f>
         <v>12</v>
       </c>
-      <c r="U11" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="V11" s="12" t="n">
-        <f aca="false">L11*Pecas!$D$18+M11*Pecas!$D$20+N11*Pecas!$D$21+O11*Pecas!$D$7+P11*Pecas!$D$13+Q11*Pecas!$D$10+R11*Pecas!$D$14+S11*Pecas!$D$15+T11*Pecas!$D$16+U11*Pecas!$D$17</f>
+      <c r="U12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="V12" s="12" t="n">
+        <f aca="false">L12*Pecas!$D$18+M12*Pecas!$D$20+N12*Pecas!$D$21+O12*Pecas!$D$7+P12*Pecas!$D$13+Q12*Pecas!$D$10+R12*Pecas!$D$14+S12*Pecas!$D$15+T12*Pecas!$D$16+U12*Pecas!$D$17</f>
         <v>9.3312</v>
       </c>
-      <c r="W11" s="13" t="n">
-        <f aca="false">L11*Pecas!$E$18+M11*Pecas!$E$20+N11*Pecas!$E$21+O11*Pecas!$E$7+P11*Pecas!$E$13+Q11*Pecas!$E$10+R11*Pecas!$E$14+S11*Pecas!$E$15+T11*Pecas!$E$16+U11*Pecas!$E$17</f>
+      <c r="W12" s="13" t="n">
+        <f aca="false">L12*Pecas!$E$18+M12*Pecas!$E$20+N12*Pecas!$E$21+O12*Pecas!$E$7+P12*Pecas!$E$13+Q12*Pecas!$E$10+R12*Pecas!$E$14+S12*Pecas!$E$15+T12*Pecas!$E$16+U12*Pecas!$E$17</f>
         <v>170.8314</v>
       </c>
-      <c r="X11" s="8" t="s">
-        <v>114</v>
+      <c r="X12" s="8" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2058,7 +2152,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -2071,40 +2165,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>69</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>90</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>93</v>
@@ -2113,25 +2207,25 @@
         <v>14</v>
       </c>
       <c r="D5" s="11" t="n">
-        <f aca="false">C5*INDEX(Modulos!$I$5:$I$11,MATCH($B5,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C5*INDEX(Modulos!$I$5:$I$12,MATCH($B5,Modulos!$A$5:$A$12,0))</f>
         <v>10626</v>
       </c>
       <c r="E5" s="13" t="n">
-        <f aca="false">C5*INDEX(Modulos!$W$5:$W$11,MATCH($B5,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C5*INDEX(Modulos!$W$5:$W$12,MATCH($B5,Modulos!$A$5:$A$12,0))</f>
         <v>4844.224</v>
       </c>
       <c r="F5" s="12" t="n">
-        <f aca="false">C5*INDEX(Modulos!$V$5:$V$11,MATCH($B5,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C5*INDEX(Modulos!$V$5:$V$12,MATCH($B5,Modulos!$A$5:$A$12,0))</f>
         <v>263.9616</v>
       </c>
       <c r="G5" s="12" t="n">
-        <f aca="false">C5*INDEX(Modulos!$I$5:$I$11,MATCH($B5,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B5,Modulos!$A$5:$A$11,0))/1000</f>
+        <f aca="false">C5*INDEX(Modulos!$I$5:$I$12,MATCH($B5,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B5,Modulos!$A$5:$A$12,0))/1000</f>
         <v>74.382</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>97</v>
@@ -2140,25 +2234,25 @@
         <v>4</v>
       </c>
       <c r="D6" s="11" t="n">
-        <f aca="false">C6*INDEX(Modulos!$I$5:$I$11,MATCH($B6,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C6*INDEX(Modulos!$I$5:$I$12,MATCH($B6,Modulos!$A$5:$A$12,0))</f>
         <v>2636</v>
       </c>
       <c r="E6" s="13" t="n">
-        <f aca="false">C6*INDEX(Modulos!$W$5:$W$11,MATCH($B6,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C6*INDEX(Modulos!$W$5:$W$12,MATCH($B6,Modulos!$A$5:$A$12,0))</f>
         <v>1217.6348</v>
       </c>
       <c r="F6" s="12" t="n">
-        <f aca="false">C6*INDEX(Modulos!$V$5:$V$11,MATCH($B6,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C6*INDEX(Modulos!$V$5:$V$12,MATCH($B6,Modulos!$A$5:$A$12,0))</f>
         <v>66.6732</v>
       </c>
       <c r="G6" s="12" t="n">
-        <f aca="false">C6*INDEX(Modulos!$I$5:$I$11,MATCH($B6,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B6,Modulos!$A$5:$A$11,0))/1000</f>
+        <f aca="false">C6*INDEX(Modulos!$I$5:$I$12,MATCH($B6,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B6,Modulos!$A$5:$A$12,0))/1000</f>
         <v>18.452</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>93</v>
@@ -2167,205 +2261,232 @@
         <v>8</v>
       </c>
       <c r="D7" s="11" t="n">
-        <f aca="false">C7*INDEX(Modulos!$I$5:$I$11,MATCH($B7,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C7*INDEX(Modulos!$I$5:$I$12,MATCH($B7,Modulos!$A$5:$A$12,0))</f>
         <v>6072</v>
       </c>
       <c r="E7" s="13" t="n">
-        <f aca="false">C7*INDEX(Modulos!$W$5:$W$11,MATCH($B7,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C7*INDEX(Modulos!$W$5:$W$12,MATCH($B7,Modulos!$A$5:$A$12,0))</f>
         <v>2768.128</v>
       </c>
       <c r="F7" s="12" t="n">
-        <f aca="false">C7*INDEX(Modulos!$V$5:$V$11,MATCH($B7,Modulos!$A$5:$A$11,0))</f>
+        <f aca="false">C7*INDEX(Modulos!$V$5:$V$12,MATCH($B7,Modulos!$A$5:$A$12,0))</f>
         <v>150.8352</v>
       </c>
       <c r="G7" s="12" t="n">
-        <f aca="false">C7*INDEX(Modulos!$I$5:$I$11,MATCH($B7,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B7,Modulos!$A$5:$A$11,0))/1000</f>
+        <f aca="false">C7*INDEX(Modulos!$I$5:$I$12,MATCH($B7,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B7,Modulos!$A$5:$A$12,0))/1000</f>
         <v>42.504</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>100</v>
       </c>
       <c r="C8" s="14" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8" s="11" t="n">
-        <f aca="false">C8*INDEX(Modulos!$I$5:$I$11,MATCH($B8,Modulos!$A$5:$A$11,0))</f>
-        <v>6831</v>
+        <f aca="false">C8*INDEX(Modulos!$I$5:$I$12,MATCH($B8,Modulos!$A$5:$A$12,0))</f>
+        <v>6072</v>
       </c>
       <c r="E8" s="13" t="n">
-        <f aca="false">C8*INDEX(Modulos!$W$5:$W$11,MATCH($B8,Modulos!$A$5:$A$11,0))</f>
-        <v>2276.424</v>
+        <f aca="false">C8*INDEX(Modulos!$W$5:$W$12,MATCH($B8,Modulos!$A$5:$A$12,0))</f>
+        <v>2023.488</v>
       </c>
       <c r="F8" s="12" t="n">
-        <f aca="false">C8*INDEX(Modulos!$V$5:$V$11,MATCH($B8,Modulos!$A$5:$A$11,0))</f>
-        <v>123.948</v>
+        <f aca="false">C8*INDEX(Modulos!$V$5:$V$12,MATCH($B8,Modulos!$A$5:$A$12,0))</f>
+        <v>110.176</v>
       </c>
       <c r="G8" s="12" t="n">
-        <f aca="false">C8*INDEX(Modulos!$I$5:$I$11,MATCH($B8,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B8,Modulos!$A$5:$A$11,0))/1000</f>
-        <v>34.155</v>
+        <f aca="false">C8*INDEX(Modulos!$I$5:$I$12,MATCH($B8,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B8,Modulos!$A$5:$A$12,0))/1000</f>
+        <v>30.36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C9" s="14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" s="11" t="n">
-        <f aca="false">C9*INDEX(Modulos!$I$5:$I$11,MATCH($B9,Modulos!$A$5:$A$11,0))</f>
-        <v>2277</v>
+        <f aca="false">C9*INDEX(Modulos!$I$5:$I$12,MATCH($B9,Modulos!$A$5:$A$12,0))</f>
+        <v>659</v>
       </c>
       <c r="E9" s="13" t="n">
-        <f aca="false">C9*INDEX(Modulos!$W$5:$W$11,MATCH($B9,Modulos!$A$5:$A$11,0))</f>
-        <v>1038.048</v>
+        <f aca="false">C9*INDEX(Modulos!$W$5:$W$12,MATCH($B9,Modulos!$A$5:$A$12,0))</f>
+        <v>223.2165</v>
       </c>
       <c r="F9" s="12" t="n">
-        <f aca="false">C9*INDEX(Modulos!$V$5:$V$11,MATCH($B9,Modulos!$A$5:$A$11,0))</f>
-        <v>56.5632</v>
+        <f aca="false">C9*INDEX(Modulos!$V$5:$V$12,MATCH($B9,Modulos!$A$5:$A$12,0))</f>
+        <v>12.2105</v>
       </c>
       <c r="G9" s="12" t="n">
-        <f aca="false">C9*INDEX(Modulos!$I$5:$I$11,MATCH($B9,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B9,Modulos!$A$5:$A$11,0))/1000</f>
-        <v>15.939</v>
+        <f aca="false">C9*INDEX(Modulos!$I$5:$I$12,MATCH($B9,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B9,Modulos!$A$5:$A$12,0))/1000</f>
+        <v>3.295</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="11" t="n">
-        <f aca="false">C10*INDEX(Modulos!$I$5:$I$11,MATCH($B10,Modulos!$A$5:$A$11,0))</f>
-        <v>1518</v>
+        <f aca="false">C10*INDEX(Modulos!$I$5:$I$12,MATCH($B10,Modulos!$A$5:$A$12,0))</f>
+        <v>2277</v>
       </c>
       <c r="E10" s="13" t="n">
-        <f aca="false">C10*INDEX(Modulos!$W$5:$W$11,MATCH($B10,Modulos!$A$5:$A$11,0))</f>
-        <v>341.6628</v>
+        <f aca="false">C10*INDEX(Modulos!$W$5:$W$12,MATCH($B10,Modulos!$A$5:$A$12,0))</f>
+        <v>1038.048</v>
       </c>
       <c r="F10" s="12" t="n">
-        <f aca="false">C10*INDEX(Modulos!$V$5:$V$11,MATCH($B10,Modulos!$A$5:$A$11,0))</f>
-        <v>18.6624</v>
+        <f aca="false">C10*INDEX(Modulos!$V$5:$V$12,MATCH($B10,Modulos!$A$5:$A$12,0))</f>
+        <v>56.5632</v>
       </c>
       <c r="G10" s="12" t="n">
-        <f aca="false">C10*INDEX(Modulos!$I$5:$I$11,MATCH($B10,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B10,Modulos!$A$5:$A$11,0))/1000</f>
-        <v>4.554</v>
+        <f aca="false">C10*INDEX(Modulos!$I$5:$I$12,MATCH($B10,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B10,Modulos!$A$5:$A$12,0))/1000</f>
+        <v>15.939</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>20</v>
+        <v>114</v>
       </c>
       <c r="C11" s="14" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D11" s="11" t="n">
-        <f aca="false">C11*INDEX(Modulos!$I$5:$I$11,MATCH($B11,Modulos!$A$5:$A$11,0))</f>
-        <v>6072</v>
+        <f aca="false">C11*INDEX(Modulos!$I$5:$I$12,MATCH($B11,Modulos!$A$5:$A$12,0))</f>
+        <v>1518</v>
       </c>
       <c r="E11" s="13" t="n">
-        <f aca="false">C11*INDEX(Modulos!$W$5:$W$11,MATCH($B11,Modulos!$A$5:$A$11,0))</f>
-        <v>1640.8208</v>
+        <f aca="false">C11*INDEX(Modulos!$W$5:$W$12,MATCH($B11,Modulos!$A$5:$A$12,0))</f>
+        <v>341.6628</v>
       </c>
       <c r="F11" s="12" t="n">
-        <f aca="false">C11*INDEX(Modulos!$V$5:$V$11,MATCH($B11,Modulos!$A$5:$A$11,0))</f>
-        <v>88.5384</v>
+        <f aca="false">C11*INDEX(Modulos!$V$5:$V$12,MATCH($B11,Modulos!$A$5:$A$12,0))</f>
+        <v>18.6624</v>
       </c>
       <c r="G11" s="12" t="n">
-        <f aca="false">C11*INDEX(Modulos!$I$5:$I$11,MATCH($B11,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B11,Modulos!$A$5:$A$11,0))/1000</f>
-        <v>18.216</v>
+        <f aca="false">C11*INDEX(Modulos!$I$5:$I$12,MATCH($B11,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B11,Modulos!$A$5:$A$12,0))/1000</f>
+        <v>4.554</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="C12" s="14" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D12" s="11" t="n">
-        <f aca="false">C12*INDEX(Modulos!$I$5:$I$11,MATCH($B12,Modulos!$A$5:$A$11,0))</f>
-        <v>3036</v>
+        <f aca="false">C12*INDEX(Modulos!$I$5:$I$12,MATCH($B12,Modulos!$A$5:$A$12,0))</f>
+        <v>6072</v>
       </c>
       <c r="E12" s="13" t="n">
-        <f aca="false">C12*INDEX(Modulos!$W$5:$W$11,MATCH($B12,Modulos!$A$5:$A$11,0))</f>
-        <v>795.2336</v>
+        <f aca="false">C12*INDEX(Modulos!$W$5:$W$12,MATCH($B12,Modulos!$A$5:$A$12,0))</f>
+        <v>1640.8208</v>
       </c>
       <c r="F12" s="12" t="n">
-        <f aca="false">C12*INDEX(Modulos!$V$5:$V$11,MATCH($B12,Modulos!$A$5:$A$11,0))</f>
-        <v>43.328</v>
+        <f aca="false">C12*INDEX(Modulos!$V$5:$V$12,MATCH($B12,Modulos!$A$5:$A$12,0))</f>
+        <v>88.5384</v>
       </c>
       <c r="G12" s="12" t="n">
-        <f aca="false">C12*INDEX(Modulos!$I$5:$I$11,MATCH($B12,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B12,Modulos!$A$5:$A$11,0))/1000</f>
-        <v>12.144</v>
+        <f aca="false">C12*INDEX(Modulos!$I$5:$I$12,MATCH($B12,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B12,Modulos!$A$5:$A$12,0))/1000</f>
+        <v>18.216</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="C13" s="14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D13" s="11" t="n">
-        <f aca="false">C13*INDEX(Modulos!$I$5:$I$11,MATCH($B13,Modulos!$A$5:$A$11,0))</f>
-        <v>3954</v>
+        <f aca="false">C13*INDEX(Modulos!$I$5:$I$12,MATCH($B13,Modulos!$A$5:$A$12,0))</f>
+        <v>3036</v>
       </c>
       <c r="E13" s="13" t="n">
-        <f aca="false">C13*INDEX(Modulos!$W$5:$W$11,MATCH($B13,Modulos!$A$5:$A$11,0))</f>
-        <v>765.0192</v>
+        <f aca="false">C13*INDEX(Modulos!$W$5:$W$12,MATCH($B13,Modulos!$A$5:$A$12,0))</f>
+        <v>795.2336</v>
       </c>
       <c r="F13" s="12" t="n">
-        <f aca="false">C13*INDEX(Modulos!$V$5:$V$11,MATCH($B13,Modulos!$A$5:$A$11,0))</f>
-        <v>42.5136</v>
+        <f aca="false">C13*INDEX(Modulos!$V$5:$V$12,MATCH($B13,Modulos!$A$5:$A$12,0))</f>
+        <v>43.328</v>
       </c>
       <c r="G13" s="12" t="n">
-        <f aca="false">C13*INDEX(Modulos!$I$5:$I$11,MATCH($B13,Modulos!$A$5:$A$11,0))*INDEX(Modulos!$H$5:$H$11,MATCH($B13,Modulos!$A$5:$A$11,0))/1000</f>
-        <v>15.816</v>
+        <f aca="false">C13*INDEX(Modulos!$I$5:$I$12,MATCH($B13,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B13,Modulos!$A$5:$A$12,0))/1000</f>
+        <v>12.144</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="4" t="n">
-        <f aca="false">SUM(C5:C13)</f>
+        <v>133</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <f aca="false">C14*INDEX(Modulos!$I$5:$I$12,MATCH($B14,Modulos!$A$5:$A$12,0))</f>
+        <v>3954</v>
+      </c>
+      <c r="E14" s="13" t="n">
+        <f aca="false">C14*INDEX(Modulos!$W$5:$W$12,MATCH($B14,Modulos!$A$5:$A$12,0))</f>
+        <v>765.0192</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <f aca="false">C14*INDEX(Modulos!$V$5:$V$12,MATCH($B14,Modulos!$A$5:$A$12,0))</f>
+        <v>42.5136</v>
+      </c>
+      <c r="G14" s="12" t="n">
+        <f aca="false">C14*INDEX(Modulos!$I$5:$I$12,MATCH($B14,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B14,Modulos!$A$5:$A$12,0))/1000</f>
+        <v>15.816</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="4" t="n">
+        <f aca="false">SUM(C5:C14)</f>
         <v>58</v>
       </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="15" t="n">
-        <f aca="false">SUM(E5:E13)</f>
-        <v>15687.1952</v>
-      </c>
-      <c r="F14" s="16" t="n">
-        <f aca="false">SUM(F5:F13)</f>
-        <v>855.0236</v>
-      </c>
-      <c r="G14" s="16" t="n">
-        <f aca="false">SUM(G5:G13)</f>
-        <v>236.162</v>
+      <c r="D15" s="10"/>
+      <c r="E15" s="15" t="n">
+        <f aca="false">SUM(E5:E14)</f>
+        <v>15657.4757</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <f aca="false">SUM(F5:F14)</f>
+        <v>853.4621</v>
+      </c>
+      <c r="G15" s="16" t="n">
+        <f aca="false">SUM(G5:G14)</f>
+        <v>235.662</v>
       </c>
     </row>
   </sheetData>
@@ -2395,12 +2516,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2408,16 +2529,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>90</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2425,7 +2546,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$O$5:$O$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),"")="200×620"))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$O$5:$O$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),"")="200×620"))</f>
         <v>24</v>
       </c>
       <c r="C5" s="12" t="n">
@@ -2445,19 +2566,19 @@
         <v>12</v>
       </c>
       <c r="B6" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$O$5:$O$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),"")="305×620"))</f>
-        <v>28</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$O$5:$O$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),"")="305×620"))</f>
+        <v>33</v>
       </c>
       <c r="C6" s="12" t="n">
         <f aca="false">B6*Pecas!$D$6</f>
-        <v>44.1588</v>
+        <v>52.0443</v>
       </c>
       <c r="D6" s="13" t="n">
         <f aca="false">B6*Pecas!$E$6</f>
-        <v>840.3388</v>
+        <v>990.3993</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2465,19 +2586,19 @@
         <v>15</v>
       </c>
       <c r="B7" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$O$5:$O$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),"")="305×725"))</f>
-        <v>242</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$O$5:$O$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),"")="305×725"))</f>
+        <v>237</v>
       </c>
       <c r="C7" s="12" t="n">
         <f aca="false">B7*Pecas!$D$7</f>
-        <v>446.2964</v>
+        <v>437.0754</v>
       </c>
       <c r="D7" s="13" t="n">
         <f aca="false">B7*Pecas!$E$7</f>
-        <v>8492.9416</v>
+        <v>8317.4676</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2485,7 +2606,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$O$5:$O$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),"")="450×725"))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$O$5:$O$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),"")="450×725"))</f>
         <v>24</v>
       </c>
       <c r="C8" s="12" t="n">
@@ -2497,7 +2618,7 @@
         <v>1242.7008</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2505,7 +2626,7 @@
         <v>21</v>
       </c>
       <c r="B9" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$Q$5:$Q$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0)=183))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$Q$5:$Q$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=183))</f>
         <v>48</v>
       </c>
       <c r="C9" s="12" t="n">
@@ -2525,7 +2646,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$Q$5:$Q$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0)=287))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$Q$5:$Q$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=287))</f>
         <v>540</v>
       </c>
       <c r="C10" s="12" t="n">
@@ -2537,7 +2658,7 @@
         <v>667.386</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2545,7 +2666,7 @@
         <v>29</v>
       </c>
       <c r="B11" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$Q$5:$Q$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0)=415))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$Q$5:$Q$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=415))</f>
         <v>48</v>
       </c>
       <c r="C11" s="12" t="n">
@@ -2557,7 +2678,7 @@
         <v>85.776</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2565,19 +2686,19 @@
         <v>33</v>
       </c>
       <c r="B12" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$P$5:$P$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$D$5:$D$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0)=617))</f>
-        <v>104</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$P$5:$P$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$D$5:$D$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=617))</f>
+        <v>114</v>
       </c>
       <c r="C12" s="12" t="n">
         <f aca="false">B12*Pecas!$D$12</f>
-        <v>14.5184</v>
+        <v>15.9144</v>
       </c>
       <c r="D12" s="13" t="n">
         <f aca="false">B12*Pecas!$E$12</f>
-        <v>276.3176</v>
+        <v>302.8866</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2585,19 +2706,19 @@
         <v>37</v>
       </c>
       <c r="B13" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$P$5:$P$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0),--(IFERROR(INDEX(Modulos!$D$5:$D$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0)=717))</f>
-        <v>536</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$P$5:$P$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$D$5:$D$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=717))</f>
+        <v>526</v>
       </c>
       <c r="C13" s="12" t="n">
         <f aca="false">B13*Pecas!$D$13</f>
-        <v>86.9392</v>
+        <v>85.3172</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">B13*Pecas!$E$13</f>
-        <v>1654.9</v>
+        <v>1624.025</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2605,7 +2726,7 @@
         <v>41</v>
       </c>
       <c r="B14" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$R$5:$R$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$R$5:$R$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
         <v>820</v>
       </c>
       <c r="C14" s="12" t="n">
@@ -2617,7 +2738,7 @@
         <v>953.332</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2625,7 +2746,7 @@
         <v>45</v>
       </c>
       <c r="B15" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$S$5:$S$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$S$5:$S$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
         <v>136</v>
       </c>
       <c r="C15" s="12" t="n">
@@ -2637,7 +2758,7 @@
         <v>202.6264</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2645,7 +2766,7 @@
         <v>49</v>
       </c>
       <c r="B16" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$T$5:$T$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$T$5:$T$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
         <v>92</v>
       </c>
       <c r="C16" s="12" t="n">
@@ -2657,7 +2778,7 @@
         <v>203.228</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2665,7 +2786,7 @@
         <v>53</v>
       </c>
       <c r="B17" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$U$5:$U$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$U$5:$U$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
         <v>232</v>
       </c>
       <c r="C17" s="12" t="n">
@@ -2683,7 +2804,7 @@
         <v>56</v>
       </c>
       <c r="B18" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$L$5:$L$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$L$5:$L$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
         <v>1272</v>
       </c>
       <c r="C18" s="12" t="n">
@@ -2695,7 +2816,7 @@
         <v>492.9</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2703,7 +2824,7 @@
         <v>63</v>
       </c>
       <c r="B19" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$M$5:$M$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$M$5:$M$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
         <v>8</v>
       </c>
       <c r="C19" s="12" t="n">
@@ -2715,7 +2836,7 @@
         <v>2.4024</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2723,7 +2844,7 @@
         <v>65</v>
       </c>
       <c r="B20" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$13,IFERROR(INDEX(Modulos!$N$5:$N$11,MATCH(Showroom!$B$5:$B$13,Modulos!$A$5:$A$11,0)),0))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$N$5:$N$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
         <v>232</v>
       </c>
       <c r="C20" s="12" t="n">
@@ -2753,27 +2874,27 @@
         <v>0</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="12" t="n">
         <f aca="false">SUM(C5:C21)</f>
-        <v>855.0236</v>
+        <v>853.4621</v>
       </c>
       <c r="D22" s="15" t="n">
         <f aca="false">SUM(D5:D21)</f>
-        <v>15687.1952</v>
+        <v>15657.4757</v>
       </c>
       <c r="E22" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>

</xml_diff>

<commit_message>
Showroom rev. 2: norte baixo sob a janela e corredor de PDV
- Norte vira parede-baixa (346·346·270, 1.030 mm) porque a janela tem
  peitoril a 1.100; nada de estrutura acima.
- Miolo ganha corredor de PDV: duas gôndolas dupla-face (parede-fundo
  costa a costa, 3 pares) com ponta nas quatro cabeceiras, corredor de
  1.400. Organização vive no corredor e transborda para o norte baixo.
- Ilhas e checkout deslocados para abrir espaço; corredores mínimos
  1.028–1.038. 74 módulos, R$ 18.310, 998 kg, 1.480 trizetas, 0 cruzeta.
- Alocação: facing múltiplo (repetição da coluna, facings extras até 4
  por SKU, reforço de Organização no norte); 3 prateleiras vazias em 364.
- plano-pecas ganha os módulos parede-baixa e gondola; dados/54 recalc.
- Doc 18 rev. 2 com planta, elevações das paredes e das 4 faces do
  corredor, compras e ancoragem. CLAUDE.md atualizado.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WcfaWwNy7qc1Kvnvnn813R
</commit_message>
<xml_diff>
--- a/dados/54-plano-pecas.xlsx
+++ b/dados/54-plano-pecas.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="157">
   <si>
     <t xml:space="preserve">Nitron Mob PDV — as peças (lista de 10/09/2026)</t>
   </si>
@@ -325,6 +325,15 @@
     <t xml:space="preserve">Parede · ajuste de canto do sul</t>
   </si>
   <si>
+    <t xml:space="preserve">parede-baixa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">346·346·270</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parede norte · sob a janela (peitoril 1.100): 1.030 de altura, 4 prateleiras, topo com produto baixo</t>
+  </si>
+  <si>
     <t xml:space="preserve">parede-fundo</t>
   </si>
   <si>
@@ -343,12 +352,15 @@
     <t xml:space="preserve">ponta</t>
   </si>
   <si>
-    <t xml:space="preserve">346·346·270</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ponta de gôndola · cabeceira das ilhas, 4 prateleiras, baias de 323</t>
   </si>
   <si>
+    <t xml:space="preserve">gondola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gôndola do corredor de PDV · dupla-face costa a costa (744 de fundo), topo aberto, 5 prateleiras</t>
+  </si>
+  <si>
     <t xml:space="preserve">450×725</t>
   </si>
   <si>
@@ -403,7 +415,7 @@
     <t xml:space="preserve">Paredão sul · ajuste de canto</t>
   </si>
   <si>
-    <t xml:space="preserve">Paredão norte · organização</t>
+    <t xml:space="preserve">Paredão norte · organização · baixo, sob a janela</t>
   </si>
   <si>
     <t xml:space="preserve">Paredão do fundo · banho e lavanderia</t>
@@ -421,7 +433,10 @@
     <t xml:space="preserve">Ilhas · 2 ilhas de 2 × 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Pontas de gôndola · 2 por ilha</t>
+    <t xml:space="preserve">Corredor de PDV · 2 gôndolas dupla-face de 3 pares</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pontas de gôndola · 2 por ilha e 2 por gôndola</t>
   </si>
   <si>
     <t xml:space="preserve">Corredor de checkout · 2 lados × 3</t>
@@ -1349,7 +1364,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:X14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -1643,14 +1658,14 @@
         <v>101</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="10" t="n">
         <f aca="false">F7+1</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>759</v>
@@ -1659,11 +1674,11 @@
         <v>372.3</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>1535</v>
+        <v>1030.1</v>
       </c>
       <c r="L7" s="10" t="n">
         <f aca="false">4*H7</f>
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M7" s="10" t="n">
         <f aca="false">IF(G7&gt;0,4,0)</f>
@@ -1674,15 +1689,15 @@
       </c>
       <c r="O7" s="10" t="n">
         <f aca="false">H7</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P7" s="10" t="n">
         <f aca="false">2*(H7+IF(G7&gt;0,1,0))</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Q7" s="10" t="n">
         <f aca="false">2*H7</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="R7" s="10" t="n">
         <f aca="false">4*1</f>
@@ -1693,19 +1708,19 @@
         <v>8</v>
       </c>
       <c r="T7" s="10" t="n">
-        <f aca="false">4*1</f>
-        <v>4</v>
+        <f aca="false">4*0</f>
+        <v>0</v>
       </c>
       <c r="U7" s="10" t="n">
         <v>4</v>
       </c>
       <c r="V7" s="12" t="n">
         <f aca="false">L7*Pecas!$D$18+M7*Pecas!$D$20+N7*Pecas!$D$21+O7*Pecas!$D$7+P7*Pecas!$D$13+Q7*Pecas!$D$10+R7*Pecas!$D$14+S7*Pecas!$D$15+T7*Pecas!$D$16+U7*Pecas!$D$17</f>
-        <v>13.772</v>
+        <v>10.832</v>
       </c>
       <c r="W7" s="13" t="n">
         <f aca="false">L7*Pecas!$E$18+M7*Pecas!$E$20+N7*Pecas!$E$21+O7*Pecas!$E$7+P7*Pecas!$E$13+Q7*Pecas!$E$10+R7*Pecas!$E$14+S7*Pecas!$E$15+T7*Pecas!$E$16+U7*Pecas!$E$17</f>
-        <v>252.936</v>
+        <v>198.8084</v>
       </c>
       <c r="X7" s="8" t="s">
         <v>102</v>
@@ -1716,16 +1731,16 @@
         <v>103</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>287</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>617</v>
+        <v>717</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>4</v>
@@ -1738,7 +1753,7 @@
         <v>5</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>659</v>
+        <v>759</v>
       </c>
       <c r="J8" s="11" t="n">
         <v>372.3</v>
@@ -1785,55 +1800,55 @@
         <v>4</v>
       </c>
       <c r="V8" s="12" t="n">
-        <f aca="false">L8*Pecas!$D$18+M8*Pecas!$D$20+N8*Pecas!$D$21+O8*Pecas!$D$6+P8*Pecas!$D$12+Q8*Pecas!$D$10+R8*Pecas!$D$14+S8*Pecas!$D$15+T8*Pecas!$D$16+U8*Pecas!$D$17</f>
-        <v>12.2105</v>
+        <f aca="false">L8*Pecas!$D$18+M8*Pecas!$D$20+N8*Pecas!$D$21+O8*Pecas!$D$7+P8*Pecas!$D$13+Q8*Pecas!$D$10+R8*Pecas!$D$14+S8*Pecas!$D$15+T8*Pecas!$D$16+U8*Pecas!$D$17</f>
+        <v>13.772</v>
       </c>
       <c r="W8" s="13" t="n">
-        <f aca="false">L8*Pecas!$E$18+M8*Pecas!$E$20+N8*Pecas!$E$21+O8*Pecas!$E$6+P8*Pecas!$E$12+Q8*Pecas!$E$10+R8*Pecas!$E$14+S8*Pecas!$E$15+T8*Pecas!$E$16+U8*Pecas!$E$17</f>
-        <v>223.2165</v>
+        <f aca="false">L8*Pecas!$E$18+M8*Pecas!$E$20+N8*Pecas!$E$21+O8*Pecas!$E$7+P8*Pecas!$E$13+Q8*Pecas!$E$10+R8*Pecas!$E$14+S8*Pecas!$E$15+T8*Pecas!$E$16+U8*Pecas!$E$17</f>
+        <v>252.936</v>
       </c>
       <c r="X8" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>287</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>717</v>
+        <v>617</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">F9+1</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>759</v>
+        <v>659</v>
       </c>
       <c r="J9" s="11" t="n">
         <v>372.3</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>1030.1</v>
+        <v>1535</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">4*H9</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="M9" s="10" t="n">
         <f aca="false">IF(G9&gt;0,4,0)</f>
@@ -1844,15 +1859,15 @@
       </c>
       <c r="O9" s="10" t="n">
         <f aca="false">H9</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P9" s="10" t="n">
         <f aca="false">2*(H9+IF(G9&gt;0,1,0))</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q9" s="10" t="n">
         <f aca="false">2*H9</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R9" s="10" t="n">
         <f aca="false">4*1</f>
@@ -1863,19 +1878,19 @@
         <v>8</v>
       </c>
       <c r="T9" s="10" t="n">
-        <f aca="false">4*0</f>
-        <v>0</v>
+        <f aca="false">4*1</f>
+        <v>4</v>
       </c>
       <c r="U9" s="10" t="n">
         <v>4</v>
       </c>
       <c r="V9" s="12" t="n">
-        <f aca="false">L9*Pecas!$D$18+M9*Pecas!$D$20+N9*Pecas!$D$21+O9*Pecas!$D$7+P9*Pecas!$D$13+Q9*Pecas!$D$10+R9*Pecas!$D$14+S9*Pecas!$D$15+T9*Pecas!$D$16+U9*Pecas!$D$17</f>
-        <v>10.832</v>
+        <f aca="false">L9*Pecas!$D$18+M9*Pecas!$D$20+N9*Pecas!$D$21+O9*Pecas!$D$6+P9*Pecas!$D$12+Q9*Pecas!$D$10+R9*Pecas!$D$14+S9*Pecas!$D$15+T9*Pecas!$D$16+U9*Pecas!$D$17</f>
+        <v>12.2105</v>
       </c>
       <c r="W9" s="13" t="n">
-        <f aca="false">L9*Pecas!$E$18+M9*Pecas!$E$20+N9*Pecas!$E$21+O9*Pecas!$E$7+P9*Pecas!$E$13+Q9*Pecas!$E$10+R9*Pecas!$E$14+S9*Pecas!$E$15+T9*Pecas!$E$16+U9*Pecas!$E$17</f>
-        <v>198.8084</v>
+        <f aca="false">L9*Pecas!$E$18+M9*Pecas!$E$20+N9*Pecas!$E$21+O9*Pecas!$E$6+P9*Pecas!$E$12+Q9*Pecas!$E$10+R9*Pecas!$E$14+S9*Pecas!$E$15+T9*Pecas!$E$16+U9*Pecas!$E$17</f>
+        <v>223.2165</v>
       </c>
       <c r="X9" s="8" t="s">
         <v>107</v>
@@ -1883,42 +1898,42 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>20</v>
+        <v>108</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>415</v>
+        <v>287</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>717</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">F10+1</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" s="11" t="n">
         <v>759</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>500.3</v>
+        <v>372.3</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>935.2</v>
+        <v>1030.1</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">4*H10</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="M10" s="10" t="n">
         <f aca="false">IF(G10&gt;0,4,0)</f>
@@ -1929,81 +1944,81 @@
       </c>
       <c r="O10" s="10" t="n">
         <f aca="false">H10</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P10" s="10" t="n">
         <f aca="false">2*(H10+IF(G10&gt;0,1,0))</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q10" s="10" t="n">
         <f aca="false">2*H10</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R10" s="10" t="n">
+        <f aca="false">4*1</f>
+        <v>4</v>
+      </c>
+      <c r="S10" s="10" t="n">
+        <f aca="false">4*2</f>
+        <v>8</v>
+      </c>
+      <c r="T10" s="10" t="n">
         <f aca="false">4*0</f>
         <v>0</v>
       </c>
-      <c r="S10" s="10" t="n">
-        <f aca="false">4*1</f>
-        <v>4</v>
-      </c>
-      <c r="T10" s="10" t="n">
-        <f aca="false">4*1</f>
-        <v>4</v>
-      </c>
       <c r="U10" s="10" t="n">
         <v>4</v>
       </c>
       <c r="V10" s="12" t="n">
-        <f aca="false">L10*Pecas!$D$18+M10*Pecas!$D$20+N10*Pecas!$D$21+O10*Pecas!$D$8+P10*Pecas!$D$13+Q10*Pecas!$D$11+R10*Pecas!$D$14+S10*Pecas!$D$15+T10*Pecas!$D$16+U10*Pecas!$D$17</f>
-        <v>11.0673</v>
+        <f aca="false">L10*Pecas!$D$18+M10*Pecas!$D$20+N10*Pecas!$D$21+O10*Pecas!$D$7+P10*Pecas!$D$13+Q10*Pecas!$D$10+R10*Pecas!$D$14+S10*Pecas!$D$15+T10*Pecas!$D$16+U10*Pecas!$D$17</f>
+        <v>10.832</v>
       </c>
       <c r="W10" s="13" t="n">
-        <f aca="false">L10*Pecas!$E$18+M10*Pecas!$E$20+N10*Pecas!$E$21+O10*Pecas!$E$8+P10*Pecas!$E$13+Q10*Pecas!$E$11+R10*Pecas!$E$14+S10*Pecas!$E$15+T10*Pecas!$E$16+U10*Pecas!$E$17</f>
-        <v>205.1026</v>
+        <f aca="false">L10*Pecas!$E$18+M10*Pecas!$E$20+N10*Pecas!$E$21+O10*Pecas!$E$7+P10*Pecas!$E$13+Q10*Pecas!$E$10+R10*Pecas!$E$14+S10*Pecas!$E$15+T10*Pecas!$E$16+U10*Pecas!$E$17</f>
+        <v>198.8084</v>
       </c>
       <c r="X10" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>11</v>
+        <v>110</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>183</v>
+        <v>287</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>617</v>
+        <v>717</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">F11+1</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>659</v>
+        <v>759</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>268.3</v>
+        <v>372.3</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>878.1</v>
+        <v>1535</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">4*H11</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="M11" s="10" t="n">
         <f aca="false">IF(G11&gt;0,4,0)</f>
@@ -2014,64 +2029,64 @@
       </c>
       <c r="O11" s="10" t="n">
         <f aca="false">H11</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P11" s="10" t="n">
         <f aca="false">2*(H11+IF(G11&gt;0,1,0))</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q11" s="10" t="n">
         <f aca="false">2*H11</f>
+        <v>10</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <f aca="false">4*1</f>
+        <v>4</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <f aca="false">4*2</f>
         <v>8</v>
       </c>
-      <c r="R11" s="10" t="n">
-        <f aca="false">4*3</f>
-        <v>12</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <f aca="false">4*0</f>
-        <v>0</v>
-      </c>
       <c r="T11" s="10" t="n">
-        <f aca="false">4*0</f>
-        <v>0</v>
+        <f aca="false">4*1</f>
+        <v>4</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>4</v>
       </c>
       <c r="V11" s="12" t="n">
-        <f aca="false">L11*Pecas!$D$18+M11*Pecas!$D$20+N11*Pecas!$D$21+O11*Pecas!$D$5+P11*Pecas!$D$12+Q11*Pecas!$D$9+R11*Pecas!$D$14+S11*Pecas!$D$15+T11*Pecas!$D$16+U11*Pecas!$D$17</f>
-        <v>7.0856</v>
+        <f aca="false">L11*Pecas!$D$18+M11*Pecas!$D$20+N11*Pecas!$D$21+O11*Pecas!$D$7+P11*Pecas!$D$13+Q11*Pecas!$D$10+R11*Pecas!$D$14+S11*Pecas!$D$15+T11*Pecas!$D$16+U11*Pecas!$D$17</f>
+        <v>13.772</v>
       </c>
       <c r="W11" s="13" t="n">
-        <f aca="false">L11*Pecas!$E$18+M11*Pecas!$E$20+N11*Pecas!$E$21+O11*Pecas!$E$5+P11*Pecas!$E$12+Q11*Pecas!$E$9+R11*Pecas!$E$14+S11*Pecas!$E$15+T11*Pecas!$E$16+U11*Pecas!$E$17</f>
-        <v>127.5032</v>
+        <f aca="false">L11*Pecas!$E$18+M11*Pecas!$E$20+N11*Pecas!$E$21+O11*Pecas!$E$7+P11*Pecas!$E$13+Q11*Pecas!$E$10+R11*Pecas!$E$14+S11*Pecas!$E$15+T11*Pecas!$E$16+U11*Pecas!$E$17</f>
+        <v>252.936</v>
       </c>
       <c r="X11" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>114</v>
+        <v>20</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>287</v>
+        <v>415</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>717</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F12" s="9" t="n">
         <v>2</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>513</v>
+        <v>0</v>
       </c>
       <c r="H12" s="10" t="n">
         <f aca="false">F12+1</f>
@@ -2081,10 +2096,10 @@
         <v>759</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>372.3</v>
+        <v>500.3</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>1607.1</v>
+        <v>935.2</v>
       </c>
       <c r="L12" s="10" t="n">
         <f aca="false">4*H12</f>
@@ -2092,7 +2107,7 @@
       </c>
       <c r="M12" s="10" t="n">
         <f aca="false">IF(G12&gt;0,4,0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N12" s="10" t="n">
         <v>4</v>
@@ -2103,7 +2118,7 @@
       </c>
       <c r="P12" s="10" t="n">
         <f aca="false">2*(H12+IF(G12&gt;0,1,0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q12" s="10" t="n">
         <f aca="false">2*H12</f>
@@ -2114,26 +2129,196 @@
         <v>0</v>
       </c>
       <c r="S12" s="10" t="n">
-        <f aca="false">4*0</f>
-        <v>0</v>
+        <f aca="false">4*1</f>
+        <v>4</v>
       </c>
       <c r="T12" s="10" t="n">
+        <f aca="false">4*1</f>
+        <v>4</v>
+      </c>
+      <c r="U12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="V12" s="12" t="n">
+        <f aca="false">L12*Pecas!$D$18+M12*Pecas!$D$20+N12*Pecas!$D$21+O12*Pecas!$D$8+P12*Pecas!$D$13+Q12*Pecas!$D$11+R12*Pecas!$D$14+S12*Pecas!$D$15+T12*Pecas!$D$16+U12*Pecas!$D$17</f>
+        <v>11.0673</v>
+      </c>
+      <c r="W12" s="13" t="n">
+        <f aca="false">L12*Pecas!$E$18+M12*Pecas!$E$20+N12*Pecas!$E$21+O12*Pecas!$E$8+P12*Pecas!$E$13+Q12*Pecas!$E$11+R12*Pecas!$E$14+S12*Pecas!$E$15+T12*Pecas!$E$16+U12*Pecas!$E$17</f>
+        <v>205.1026</v>
+      </c>
+      <c r="X12" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>183</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>617</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <f aca="false">F13+1</f>
+        <v>4</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>659</v>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>268.3</v>
+      </c>
+      <c r="K13" s="11" t="n">
+        <v>878.1</v>
+      </c>
+      <c r="L13" s="10" t="n">
+        <f aca="false">4*H13</f>
+        <v>16</v>
+      </c>
+      <c r="M13" s="10" t="n">
+        <f aca="false">IF(G13&gt;0,4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N13" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="O13" s="10" t="n">
+        <f aca="false">H13</f>
+        <v>4</v>
+      </c>
+      <c r="P13" s="10" t="n">
+        <f aca="false">2*(H13+IF(G13&gt;0,1,0))</f>
+        <v>8</v>
+      </c>
+      <c r="Q13" s="10" t="n">
+        <f aca="false">2*H13</f>
+        <v>8</v>
+      </c>
+      <c r="R13" s="10" t="n">
         <f aca="false">4*3</f>
         <v>12</v>
       </c>
-      <c r="U12" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="V12" s="12" t="n">
-        <f aca="false">L12*Pecas!$D$18+M12*Pecas!$D$20+N12*Pecas!$D$21+O12*Pecas!$D$7+P12*Pecas!$D$13+Q12*Pecas!$D$10+R12*Pecas!$D$14+S12*Pecas!$D$15+T12*Pecas!$D$16+U12*Pecas!$D$17</f>
+      <c r="S13" s="10" t="n">
+        <f aca="false">4*0</f>
+        <v>0</v>
+      </c>
+      <c r="T13" s="10" t="n">
+        <f aca="false">4*0</f>
+        <v>0</v>
+      </c>
+      <c r="U13" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="V13" s="12" t="n">
+        <f aca="false">L13*Pecas!$D$18+M13*Pecas!$D$20+N13*Pecas!$D$21+O13*Pecas!$D$5+P13*Pecas!$D$12+Q13*Pecas!$D$9+R13*Pecas!$D$14+S13*Pecas!$D$15+T13*Pecas!$D$16+U13*Pecas!$D$17</f>
+        <v>7.0856</v>
+      </c>
+      <c r="W13" s="13" t="n">
+        <f aca="false">L13*Pecas!$E$18+M13*Pecas!$E$20+N13*Pecas!$E$21+O13*Pecas!$E$5+P13*Pecas!$E$12+Q13*Pecas!$E$9+R13*Pecas!$E$14+S13*Pecas!$E$15+T13*Pecas!$E$16+U13*Pecas!$E$17</f>
+        <v>127.5032</v>
+      </c>
+      <c r="X13" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>287</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>717</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>513</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <f aca="false">F14+1</f>
+        <v>3</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>759</v>
+      </c>
+      <c r="J14" s="11" t="n">
+        <v>372.3</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>1607.1</v>
+      </c>
+      <c r="L14" s="10" t="n">
+        <f aca="false">4*H14</f>
+        <v>12</v>
+      </c>
+      <c r="M14" s="10" t="n">
+        <f aca="false">IF(G14&gt;0,4,0)</f>
+        <v>4</v>
+      </c>
+      <c r="N14" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="O14" s="10" t="n">
+        <f aca="false">H14</f>
+        <v>3</v>
+      </c>
+      <c r="P14" s="10" t="n">
+        <f aca="false">2*(H14+IF(G14&gt;0,1,0))</f>
+        <v>8</v>
+      </c>
+      <c r="Q14" s="10" t="n">
+        <f aca="false">2*H14</f>
+        <v>6</v>
+      </c>
+      <c r="R14" s="10" t="n">
+        <f aca="false">4*0</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="10" t="n">
+        <f aca="false">4*0</f>
+        <v>0</v>
+      </c>
+      <c r="T14" s="10" t="n">
+        <f aca="false">4*3</f>
+        <v>12</v>
+      </c>
+      <c r="U14" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="V14" s="12" t="n">
+        <f aca="false">L14*Pecas!$D$18+M14*Pecas!$D$20+N14*Pecas!$D$21+O14*Pecas!$D$7+P14*Pecas!$D$13+Q14*Pecas!$D$10+R14*Pecas!$D$14+S14*Pecas!$D$15+T14*Pecas!$D$16+U14*Pecas!$D$17</f>
         <v>9.3312</v>
       </c>
-      <c r="W12" s="13" t="n">
-        <f aca="false">L12*Pecas!$E$18+M12*Pecas!$E$20+N12*Pecas!$E$21+O12*Pecas!$E$7+P12*Pecas!$E$13+Q12*Pecas!$E$10+R12*Pecas!$E$14+S12*Pecas!$E$15+T12*Pecas!$E$16+U12*Pecas!$E$17</f>
+      <c r="W14" s="13" t="n">
+        <f aca="false">L14*Pecas!$E$18+M14*Pecas!$E$20+N14*Pecas!$E$21+O14*Pecas!$E$7+P14*Pecas!$E$13+Q14*Pecas!$E$10+R14*Pecas!$E$14+S14*Pecas!$E$15+T14*Pecas!$E$16+U14*Pecas!$E$17</f>
         <v>170.8314</v>
       </c>
-      <c r="X12" s="8" t="s">
-        <v>116</v>
+      <c r="X14" s="8" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2152,7 +2337,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -2165,40 +2350,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>69</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>90</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>93</v>
@@ -2207,25 +2392,25 @@
         <v>14</v>
       </c>
       <c r="D5" s="11" t="n">
-        <f aca="false">C5*INDEX(Modulos!$I$5:$I$12,MATCH($B5,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C5*INDEX(Modulos!$I$5:$I$14,MATCH($B5,Modulos!$A$5:$A$14,0))</f>
         <v>10626</v>
       </c>
       <c r="E5" s="13" t="n">
-        <f aca="false">C5*INDEX(Modulos!$W$5:$W$12,MATCH($B5,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C5*INDEX(Modulos!$W$5:$W$14,MATCH($B5,Modulos!$A$5:$A$14,0))</f>
         <v>4844.224</v>
       </c>
       <c r="F5" s="12" t="n">
-        <f aca="false">C5*INDEX(Modulos!$V$5:$V$12,MATCH($B5,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C5*INDEX(Modulos!$V$5:$V$14,MATCH($B5,Modulos!$A$5:$A$14,0))</f>
         <v>263.9616</v>
       </c>
       <c r="G5" s="12" t="n">
-        <f aca="false">C5*INDEX(Modulos!$I$5:$I$12,MATCH($B5,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B5,Modulos!$A$5:$A$12,0))/1000</f>
+        <f aca="false">C5*INDEX(Modulos!$I$5:$I$14,MATCH($B5,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B5,Modulos!$A$5:$A$14,0))/1000</f>
         <v>74.382</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>97</v>
@@ -2234,106 +2419,106 @@
         <v>4</v>
       </c>
       <c r="D6" s="11" t="n">
-        <f aca="false">C6*INDEX(Modulos!$I$5:$I$12,MATCH($B6,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C6*INDEX(Modulos!$I$5:$I$14,MATCH($B6,Modulos!$A$5:$A$14,0))</f>
         <v>2636</v>
       </c>
       <c r="E6" s="13" t="n">
-        <f aca="false">C6*INDEX(Modulos!$W$5:$W$12,MATCH($B6,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C6*INDEX(Modulos!$W$5:$W$14,MATCH($B6,Modulos!$A$5:$A$14,0))</f>
         <v>1217.6348</v>
       </c>
       <c r="F6" s="12" t="n">
-        <f aca="false">C6*INDEX(Modulos!$V$5:$V$12,MATCH($B6,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C6*INDEX(Modulos!$V$5:$V$14,MATCH($B6,Modulos!$A$5:$A$14,0))</f>
         <v>66.6732</v>
       </c>
       <c r="G6" s="12" t="n">
-        <f aca="false">C6*INDEX(Modulos!$I$5:$I$12,MATCH($B6,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B6,Modulos!$A$5:$A$12,0))/1000</f>
+        <f aca="false">C6*INDEX(Modulos!$I$5:$I$14,MATCH($B6,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B6,Modulos!$A$5:$A$14,0))/1000</f>
         <v>18.452</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="C7" s="14" t="n">
         <v>8</v>
       </c>
       <c r="D7" s="11" t="n">
-        <f aca="false">C7*INDEX(Modulos!$I$5:$I$12,MATCH($B7,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C7*INDEX(Modulos!$I$5:$I$14,MATCH($B7,Modulos!$A$5:$A$14,0))</f>
         <v>6072</v>
       </c>
       <c r="E7" s="13" t="n">
-        <f aca="false">C7*INDEX(Modulos!$W$5:$W$12,MATCH($B7,Modulos!$A$5:$A$12,0))</f>
-        <v>2768.128</v>
+        <f aca="false">C7*INDEX(Modulos!$W$5:$W$14,MATCH($B7,Modulos!$A$5:$A$14,0))</f>
+        <v>1590.4672</v>
       </c>
       <c r="F7" s="12" t="n">
-        <f aca="false">C7*INDEX(Modulos!$V$5:$V$12,MATCH($B7,Modulos!$A$5:$A$12,0))</f>
-        <v>150.8352</v>
+        <f aca="false">C7*INDEX(Modulos!$V$5:$V$14,MATCH($B7,Modulos!$A$5:$A$14,0))</f>
+        <v>86.656</v>
       </c>
       <c r="G7" s="12" t="n">
-        <f aca="false">C7*INDEX(Modulos!$I$5:$I$12,MATCH($B7,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B7,Modulos!$A$5:$A$12,0))/1000</f>
-        <v>42.504</v>
+        <f aca="false">C7*INDEX(Modulos!$I$5:$I$14,MATCH($B7,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B7,Modulos!$A$5:$A$14,0))/1000</f>
+        <v>24.288</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>8</v>
       </c>
       <c r="D8" s="11" t="n">
-        <f aca="false">C8*INDEX(Modulos!$I$5:$I$12,MATCH($B8,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C8*INDEX(Modulos!$I$5:$I$14,MATCH($B8,Modulos!$A$5:$A$14,0))</f>
         <v>6072</v>
       </c>
       <c r="E8" s="13" t="n">
-        <f aca="false">C8*INDEX(Modulos!$W$5:$W$12,MATCH($B8,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C8*INDEX(Modulos!$W$5:$W$14,MATCH($B8,Modulos!$A$5:$A$14,0))</f>
         <v>2023.488</v>
       </c>
       <c r="F8" s="12" t="n">
-        <f aca="false">C8*INDEX(Modulos!$V$5:$V$12,MATCH($B8,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C8*INDEX(Modulos!$V$5:$V$14,MATCH($B8,Modulos!$A$5:$A$14,0))</f>
         <v>110.176</v>
       </c>
       <c r="G8" s="12" t="n">
-        <f aca="false">C8*INDEX(Modulos!$I$5:$I$12,MATCH($B8,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B8,Modulos!$A$5:$A$12,0))/1000</f>
+        <f aca="false">C8*INDEX(Modulos!$I$5:$I$14,MATCH($B8,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B8,Modulos!$A$5:$A$14,0))/1000</f>
         <v>30.36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="11" t="n">
-        <f aca="false">C9*INDEX(Modulos!$I$5:$I$12,MATCH($B9,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C9*INDEX(Modulos!$I$5:$I$14,MATCH($B9,Modulos!$A$5:$A$14,0))</f>
         <v>659</v>
       </c>
       <c r="E9" s="13" t="n">
-        <f aca="false">C9*INDEX(Modulos!$W$5:$W$12,MATCH($B9,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C9*INDEX(Modulos!$W$5:$W$14,MATCH($B9,Modulos!$A$5:$A$14,0))</f>
         <v>223.2165</v>
       </c>
       <c r="F9" s="12" t="n">
-        <f aca="false">C9*INDEX(Modulos!$V$5:$V$12,MATCH($B9,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C9*INDEX(Modulos!$V$5:$V$14,MATCH($B9,Modulos!$A$5:$A$14,0))</f>
         <v>12.2105</v>
       </c>
       <c r="G9" s="12" t="n">
-        <f aca="false">C9*INDEX(Modulos!$I$5:$I$12,MATCH($B9,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B9,Modulos!$A$5:$A$12,0))/1000</f>
+        <f aca="false">C9*INDEX(Modulos!$I$5:$I$14,MATCH($B9,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B9,Modulos!$A$5:$A$14,0))/1000</f>
         <v>3.295</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>93</v>
@@ -2342,52 +2527,52 @@
         <v>3</v>
       </c>
       <c r="D10" s="11" t="n">
-        <f aca="false">C10*INDEX(Modulos!$I$5:$I$12,MATCH($B10,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C10*INDEX(Modulos!$I$5:$I$14,MATCH($B10,Modulos!$A$5:$A$14,0))</f>
         <v>2277</v>
       </c>
       <c r="E10" s="13" t="n">
-        <f aca="false">C10*INDEX(Modulos!$W$5:$W$12,MATCH($B10,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C10*INDEX(Modulos!$W$5:$W$14,MATCH($B10,Modulos!$A$5:$A$14,0))</f>
         <v>1038.048</v>
       </c>
       <c r="F10" s="12" t="n">
-        <f aca="false">C10*INDEX(Modulos!$V$5:$V$12,MATCH($B10,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C10*INDEX(Modulos!$V$5:$V$14,MATCH($B10,Modulos!$A$5:$A$14,0))</f>
         <v>56.5632</v>
       </c>
       <c r="G10" s="12" t="n">
-        <f aca="false">C10*INDEX(Modulos!$I$5:$I$12,MATCH($B10,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B10,Modulos!$A$5:$A$12,0))/1000</f>
+        <f aca="false">C10*INDEX(Modulos!$I$5:$I$14,MATCH($B10,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B10,Modulos!$A$5:$A$14,0))/1000</f>
         <v>15.939</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C11" s="14" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="11" t="n">
-        <f aca="false">C11*INDEX(Modulos!$I$5:$I$12,MATCH($B11,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C11*INDEX(Modulos!$I$5:$I$14,MATCH($B11,Modulos!$A$5:$A$14,0))</f>
         <v>1518</v>
       </c>
       <c r="E11" s="13" t="n">
-        <f aca="false">C11*INDEX(Modulos!$W$5:$W$12,MATCH($B11,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C11*INDEX(Modulos!$W$5:$W$14,MATCH($B11,Modulos!$A$5:$A$14,0))</f>
         <v>341.6628</v>
       </c>
       <c r="F11" s="12" t="n">
-        <f aca="false">C11*INDEX(Modulos!$V$5:$V$12,MATCH($B11,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C11*INDEX(Modulos!$V$5:$V$14,MATCH($B11,Modulos!$A$5:$A$14,0))</f>
         <v>18.6624</v>
       </c>
       <c r="G11" s="12" t="n">
-        <f aca="false">C11*INDEX(Modulos!$I$5:$I$12,MATCH($B11,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B11,Modulos!$A$5:$A$12,0))/1000</f>
+        <f aca="false">C11*INDEX(Modulos!$I$5:$I$14,MATCH($B11,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B11,Modulos!$A$5:$A$14,0))/1000</f>
         <v>4.554</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>20</v>
@@ -2396,97 +2581,124 @@
         <v>8</v>
       </c>
       <c r="D12" s="11" t="n">
-        <f aca="false">C12*INDEX(Modulos!$I$5:$I$12,MATCH($B12,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C12*INDEX(Modulos!$I$5:$I$14,MATCH($B12,Modulos!$A$5:$A$14,0))</f>
         <v>6072</v>
       </c>
       <c r="E12" s="13" t="n">
-        <f aca="false">C12*INDEX(Modulos!$W$5:$W$12,MATCH($B12,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C12*INDEX(Modulos!$W$5:$W$14,MATCH($B12,Modulos!$A$5:$A$14,0))</f>
         <v>1640.8208</v>
       </c>
       <c r="F12" s="12" t="n">
-        <f aca="false">C12*INDEX(Modulos!$V$5:$V$12,MATCH($B12,Modulos!$A$5:$A$12,0))</f>
+        <f aca="false">C12*INDEX(Modulos!$V$5:$V$14,MATCH($B12,Modulos!$A$5:$A$14,0))</f>
         <v>88.5384</v>
       </c>
       <c r="G12" s="12" t="n">
-        <f aca="false">C12*INDEX(Modulos!$I$5:$I$12,MATCH($B12,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B12,Modulos!$A$5:$A$12,0))/1000</f>
+        <f aca="false">C12*INDEX(Modulos!$I$5:$I$14,MATCH($B12,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B12,Modulos!$A$5:$A$14,0))/1000</f>
         <v>18.216</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C13" s="14" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D13" s="11" t="n">
-        <f aca="false">C13*INDEX(Modulos!$I$5:$I$12,MATCH($B13,Modulos!$A$5:$A$12,0))</f>
-        <v>3036</v>
+        <f aca="false">C13*INDEX(Modulos!$I$5:$I$14,MATCH($B13,Modulos!$A$5:$A$14,0))</f>
+        <v>9108</v>
       </c>
       <c r="E13" s="13" t="n">
-        <f aca="false">C13*INDEX(Modulos!$W$5:$W$12,MATCH($B13,Modulos!$A$5:$A$12,0))</f>
-        <v>795.2336</v>
+        <f aca="false">C13*INDEX(Modulos!$W$5:$W$14,MATCH($B13,Modulos!$A$5:$A$14,0))</f>
+        <v>3035.232</v>
       </c>
       <c r="F13" s="12" t="n">
-        <f aca="false">C13*INDEX(Modulos!$V$5:$V$12,MATCH($B13,Modulos!$A$5:$A$12,0))</f>
-        <v>43.328</v>
+        <f aca="false">C13*INDEX(Modulos!$V$5:$V$14,MATCH($B13,Modulos!$A$5:$A$14,0))</f>
+        <v>165.264</v>
       </c>
       <c r="G13" s="12" t="n">
-        <f aca="false">C13*INDEX(Modulos!$I$5:$I$12,MATCH($B13,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B13,Modulos!$A$5:$A$12,0))/1000</f>
-        <v>12.144</v>
+        <f aca="false">C13*INDEX(Modulos!$I$5:$I$14,MATCH($B13,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B13,Modulos!$A$5:$A$14,0))/1000</f>
+        <v>45.54</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="C14" s="14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D14" s="11" t="n">
-        <f aca="false">C14*INDEX(Modulos!$I$5:$I$12,MATCH($B14,Modulos!$A$5:$A$12,0))</f>
-        <v>3954</v>
+        <f aca="false">C14*INDEX(Modulos!$I$5:$I$14,MATCH($B14,Modulos!$A$5:$A$14,0))</f>
+        <v>6072</v>
       </c>
       <c r="E14" s="13" t="n">
-        <f aca="false">C14*INDEX(Modulos!$W$5:$W$12,MATCH($B14,Modulos!$A$5:$A$12,0))</f>
-        <v>765.0192</v>
+        <f aca="false">C14*INDEX(Modulos!$W$5:$W$14,MATCH($B14,Modulos!$A$5:$A$14,0))</f>
+        <v>1590.4672</v>
       </c>
       <c r="F14" s="12" t="n">
-        <f aca="false">C14*INDEX(Modulos!$V$5:$V$12,MATCH($B14,Modulos!$A$5:$A$12,0))</f>
-        <v>42.5136</v>
+        <f aca="false">C14*INDEX(Modulos!$V$5:$V$14,MATCH($B14,Modulos!$A$5:$A$14,0))</f>
+        <v>86.656</v>
       </c>
       <c r="G14" s="12" t="n">
-        <f aca="false">C14*INDEX(Modulos!$I$5:$I$12,MATCH($B14,Modulos!$A$5:$A$12,0))*INDEX(Modulos!$H$5:$H$12,MATCH($B14,Modulos!$A$5:$A$12,0))/1000</f>
-        <v>15.816</v>
+        <f aca="false">C14*INDEX(Modulos!$I$5:$I$14,MATCH($B14,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B14,Modulos!$A$5:$A$14,0))/1000</f>
+        <v>24.288</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="4" t="n">
-        <f aca="false">SUM(C5:C14)</f>
-        <v>58</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="15" t="n">
-        <f aca="false">SUM(E5:E14)</f>
-        <v>15657.4757</v>
-      </c>
-      <c r="F15" s="16" t="n">
-        <f aca="false">SUM(F5:F14)</f>
-        <v>853.4621</v>
-      </c>
-      <c r="G15" s="16" t="n">
-        <f aca="false">SUM(G5:G14)</f>
-        <v>235.662</v>
+        <v>138</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <f aca="false">C15*INDEX(Modulos!$I$5:$I$14,MATCH($B15,Modulos!$A$5:$A$14,0))</f>
+        <v>3954</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <f aca="false">C15*INDEX(Modulos!$W$5:$W$14,MATCH($B15,Modulos!$A$5:$A$14,0))</f>
+        <v>765.0192</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <f aca="false">C15*INDEX(Modulos!$V$5:$V$14,MATCH($B15,Modulos!$A$5:$A$14,0))</f>
+        <v>42.5136</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <f aca="false">C15*INDEX(Modulos!$I$5:$I$14,MATCH($B15,Modulos!$A$5:$A$14,0))*INDEX(Modulos!$H$5:$H$14,MATCH($B15,Modulos!$A$5:$A$14,0))/1000</f>
+        <v>15.816</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B16" s="10"/>
+      <c r="C16" s="4" t="n">
+        <f aca="false">SUM(C5:C15)</f>
+        <v>74</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="15" t="n">
+        <f aca="false">SUM(E5:E15)</f>
+        <v>18310.2805</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <f aca="false">SUM(F5:F15)</f>
+        <v>997.8749</v>
+      </c>
+      <c r="G16" s="16" t="n">
+        <f aca="false">SUM(G5:G15)</f>
+        <v>275.13</v>
       </c>
     </row>
   </sheetData>
@@ -2516,12 +2728,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2529,16 +2741,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>90</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2546,7 +2758,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$O$5:$O$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),"")="200×620"))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$O$5:$O$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),"")="200×620"))</f>
         <v>24</v>
       </c>
       <c r="C5" s="12" t="n">
@@ -2566,7 +2778,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$O$5:$O$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),"")="305×620"))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$O$5:$O$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),"")="305×620"))</f>
         <v>33</v>
       </c>
       <c r="C6" s="12" t="n">
@@ -2578,7 +2790,7 @@
         <v>990.3993</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2586,19 +2798,19 @@
         <v>15</v>
       </c>
       <c r="B7" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$O$5:$O$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),"")="305×725"))</f>
-        <v>237</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$O$5:$O$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),"")="305×725"))</f>
+        <v>289</v>
       </c>
       <c r="C7" s="12" t="n">
         <f aca="false">B7*Pecas!$D$7</f>
-        <v>437.0754</v>
+        <v>532.9738</v>
       </c>
       <c r="D7" s="13" t="n">
         <f aca="false">B7*Pecas!$E$7</f>
-        <v>8317.4676</v>
+        <v>10142.3972</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2606,7 +2818,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$O$5:$O$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),"")="450×725"))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$O$5:$O$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$B$5:$B$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),"")="450×725"))</f>
         <v>24</v>
       </c>
       <c r="C8" s="12" t="n">
@@ -2618,7 +2830,7 @@
         <v>1242.7008</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2626,7 +2838,7 @@
         <v>21</v>
       </c>
       <c r="B9" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$Q$5:$Q$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=183))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$Q$5:$Q$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0)=183))</f>
         <v>48</v>
       </c>
       <c r="C9" s="12" t="n">
@@ -2646,19 +2858,19 @@
         <v>25</v>
       </c>
       <c r="B10" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$Q$5:$Q$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=287))</f>
-        <v>540</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$Q$5:$Q$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0)=287))</f>
+        <v>644</v>
       </c>
       <c r="C10" s="12" t="n">
         <f aca="false">B10*Pecas!$D$10</f>
-        <v>35.046</v>
+        <v>41.7956</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">B10*Pecas!$E$10</f>
-        <v>667.386</v>
+        <v>795.9196</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2666,7 +2878,7 @@
         <v>29</v>
       </c>
       <c r="B11" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$Q$5:$Q$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=415))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$Q$5:$Q$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$C$5:$C$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0)=415))</f>
         <v>48</v>
       </c>
       <c r="C11" s="12" t="n">
@@ -2678,7 +2890,7 @@
         <v>85.776</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2686,7 +2898,7 @@
         <v>33</v>
       </c>
       <c r="B12" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$P$5:$P$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$D$5:$D$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=617))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$P$5:$P$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$D$5:$D$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0)=617))</f>
         <v>114</v>
       </c>
       <c r="C12" s="12" t="n">
@@ -2698,7 +2910,7 @@
         <v>302.8866</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2706,19 +2918,19 @@
         <v>37</v>
       </c>
       <c r="B13" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$P$5:$P$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0),--(IFERROR(INDEX(Modulos!$D$5:$D$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0)=717))</f>
-        <v>526</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$P$5:$P$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0),--(IFERROR(INDEX(Modulos!$D$5:$D$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0)=717))</f>
+        <v>630</v>
       </c>
       <c r="C13" s="12" t="n">
         <f aca="false">B13*Pecas!$D$13</f>
-        <v>85.3172</v>
+        <v>102.186</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">B13*Pecas!$E$13</f>
-        <v>1624.025</v>
+        <v>1945.125</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2726,19 +2938,19 @@
         <v>41</v>
       </c>
       <c r="B14" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$R$5:$R$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
-        <v>820</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$R$5:$R$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0))</f>
+        <v>724</v>
       </c>
       <c r="C14" s="12" t="n">
         <f aca="false">B14*Pecas!$D$14</f>
-        <v>50.102</v>
+        <v>44.2364</v>
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">B14*Pecas!$E$14</f>
-        <v>953.332</v>
+        <v>841.7224</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2746,19 +2958,19 @@
         <v>45</v>
       </c>
       <c r="B15" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$S$5:$S$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
-        <v>136</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$S$5:$S$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0))</f>
+        <v>328</v>
       </c>
       <c r="C15" s="12" t="n">
         <f aca="false">B15*Pecas!$D$15</f>
-        <v>10.6488</v>
+        <v>25.6824</v>
       </c>
       <c r="D15" s="13" t="n">
         <f aca="false">B15*Pecas!$E$15</f>
-        <v>202.6264</v>
+        <v>488.6872</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2766,19 +2978,19 @@
         <v>49</v>
       </c>
       <c r="B16" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$T$5:$T$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
-        <v>92</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$T$5:$T$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0))</f>
+        <v>140</v>
       </c>
       <c r="C16" s="12" t="n">
         <f aca="false">B16*Pecas!$D$16</f>
-        <v>10.6812</v>
+        <v>16.254</v>
       </c>
       <c r="D16" s="13" t="n">
         <f aca="false">B16*Pecas!$E$16</f>
-        <v>203.228</v>
+        <v>309.26</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2786,16 +2998,16 @@
         <v>53</v>
       </c>
       <c r="B17" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$U$5:$U$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
-        <v>232</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$U$5:$U$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0))</f>
+        <v>296</v>
       </c>
       <c r="C17" s="12" t="n">
         <f aca="false">B17*Pecas!$D$17</f>
-        <v>3.1552</v>
+        <v>4.0256</v>
       </c>
       <c r="D17" s="13" t="n">
         <f aca="false">B17*Pecas!$E$17</f>
-        <v>59.9488</v>
+        <v>76.4864</v>
       </c>
       <c r="E17" s="8"/>
     </row>
@@ -2804,19 +3016,19 @@
         <v>56</v>
       </c>
       <c r="B18" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$L$5:$L$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
-        <v>1272</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$L$5:$L$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0))</f>
+        <v>1480</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">B18*Pecas!$D$18</f>
-        <v>56.3496</v>
+        <v>65.564</v>
       </c>
       <c r="D18" s="13" t="n">
         <f aca="false">B18*Pecas!$E$18</f>
-        <v>492.9</v>
+        <v>573.5</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2824,7 +3036,7 @@
         <v>63</v>
       </c>
       <c r="B19" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$M$5:$M$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$M$5:$M$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0))</f>
         <v>8</v>
       </c>
       <c r="C19" s="12" t="n">
@@ -2836,7 +3048,7 @@
         <v>2.4024</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2844,16 +3056,16 @@
         <v>65</v>
       </c>
       <c r="B20" s="11" t="n">
-        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$14,IFERROR(INDEX(Modulos!$N$5:$N$12,MATCH(Showroom!$B$5:$B$14,Modulos!$A$5:$A$12,0)),0))</f>
-        <v>232</v>
+        <f aca="false">SUMPRODUCT(Showroom!$C$5:$C$15,IFERROR(INDEX(Modulos!$N$5:$N$14,MATCH(Showroom!$B$5:$B$15,Modulos!$A$5:$A$14,0)),0))</f>
+        <v>296</v>
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">B20*Pecas!$D$21</f>
-        <v>0.2552</v>
+        <v>0.3256</v>
       </c>
       <c r="D20" s="13" t="n">
         <f aca="false">B20*Pecas!$E$21</f>
-        <v>2.2504</v>
+        <v>2.8712</v>
       </c>
       <c r="E20" s="8"/>
     </row>
@@ -2874,27 +3086,27 @@
         <v>0</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="12" t="n">
         <f aca="false">SUM(C5:C21)</f>
-        <v>853.4621</v>
+        <v>997.8749</v>
       </c>
       <c r="D22" s="15" t="n">
         <f aca="false">SUM(D5:D21)</f>
-        <v>15657.4757</v>
+        <v>18310.2805</v>
       </c>
       <c r="E22" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>

</xml_diff>